<commit_message>
Rev B / rev A order: 10 uF CL31B106KAHZW6E, beads BLM31PG391SN1L
Both earlier substitutes (CL31B106KAHNNNE, BLM31KN102SH1L) are on
backorder at Mouser. CL31B106KAHZW6E has the same rating (1.4 mm tall).
The isolated-supply beads need no 1 kOhm: TI's reference uses 330 Ohm;
BLM31PG391SN1L is 390 Ohm @ 100 MHz, 2 A, 50 mOhm. Field-only changes;
order lists regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -400,7 +400,7 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL31B106KAHNNNE</t>
+          <t xml:space="preserve">CL31B106KAHZW6E</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1590,7 +1590,7 @@
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLM31KN102SH1L</t>
+          <t xml:space="preserve">BLM31PG391SN1L</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLM31KN102SH1L [CC8 SE4]</t>
+          <t xml:space="preserve">BLM31PG391SN1L [CC8 SE4]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rev A: can-ssr display not fitted; rev B display to-do
The MAX7219 is obsolete and expensive, so rev A can-ssr boards are built
without U40 and the parts that only serve it (U41, D40/D41, R50, C43/C44).
tools/order_bom.py gains a per-revision NOT_FITTED list; rev A order lists
regenerated (118 lines, 443 parts). docs/rev-b-changes.md: replace the
display, I2C OLED (with burn-in handling) or HT16K33.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -174,11 +174,11 @@
         </is>
       </c>
       <c r="D7">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">100nF 50V X7R [CO20 CC8 IO7 SE5 SS17]</t>
+          <t xml:space="preserve">100nF 50V X7R [CO20 CC8 IO7 SE5 SS16]</t>
         </is>
       </c>
     </row>
@@ -409,11 +409,11 @@
         </is>
       </c>
       <c r="D17">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">10uF 25V X7R [CO7 CC12 IO3 SE8 SS6]</t>
+          <t xml:space="preserve">10uF 25V X7R [CO7 CC12 IO3 SE8 SS5]</t>
         </is>
       </c>
     </row>
@@ -908,114 +908,114 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC1206FR-0727KL</t>
-        </is>
-      </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-0727KL</t>
+          <t xml:space="preserve">C0805C270J5GACTU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">KEMET</t>
         </is>
       </c>
       <c r="D38">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">27k [SS1]</t>
+          <t xml:space="preserve">27pF 50V C0G [CO4 SS2]</t>
         </is>
       </c>
     </row>
     <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">652-MF-MSMF200/16X-2</t>
+        </is>
+      </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">C0805C270J5GACTU</t>
+          <t xml:space="preserve">MF-MSMF200/16X-2</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t xml:space="preserve">KEMET</t>
+          <t xml:space="preserve">Bourns</t>
         </is>
       </c>
       <c r="D39">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">27pF 50V C0G [CO4 SS2]</t>
+          <t xml:space="preserve">2A [CC1]</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">652-MF-MSMF200/16X-2</t>
+          <t xml:space="preserve">863-2N7002LT1G</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">MF-MSMF200/16X-2</t>
+          <t xml:space="preserve">2N7002LT1G</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bourns</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="D40">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">2A [CC1]</t>
+          <t xml:space="preserve">2N7002 [SS5]</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">863-2N7002LT1G</t>
+          <t xml:space="preserve">187-CL31B335KAHVPNE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2N7002LT1G</t>
+          <t xml:space="preserve">CL31B335KAHVPNE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t xml:space="preserve">onsemi</t>
+          <t xml:space="preserve">Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="D41">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2N7002 [SS5]</t>
+          <t xml:space="preserve">3.3uF 25V X7R [CO1]</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">187-CL31B335KAHVPNE</t>
+          <t xml:space="preserve">603-RC1206FR-07300RL</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL31B335KAHVPNE</t>
+          <t xml:space="preserve">RC1206FR-07300RL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samsung Electro-Mechanics</t>
+          <t xml:space="preserve">Yageo</t>
         </is>
       </c>
       <c r="D42">
@@ -1023,44 +1023,44 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.3uF 25V X7R [CO1]</t>
+          <t xml:space="preserve">300R [CO1]</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC1206FR-07300RL</t>
-        </is>
-      </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-07300RL</t>
+          <t xml:space="preserve">RMCF1206FT330R</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">Stackpole</t>
         </is>
       </c>
       <c r="D43">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">300R [CO1]</t>
+          <t xml:space="preserve">330R [CO2 IO4]</t>
         </is>
       </c>
     </row>
     <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603-RC1206FR-07332KL</t>
+        </is>
+      </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">RMCF1206FT330R</t>
+          <t xml:space="preserve">RC1206FR-07332KL</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stackpole</t>
+          <t xml:space="preserve">Yageo</t>
         </is>
       </c>
       <c r="D44">
@@ -1068,19 +1068,19 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">330R [CO2 IO4]</t>
+          <t xml:space="preserve">332k [SS6]</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-RC1206FR-07332KL</t>
+          <t xml:space="preserve">603-RC1206FR-074K7L</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-07332KL</t>
+          <t xml:space="preserve">RC1206FR-074K7L</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1089,68 +1089,68 @@
         </is>
       </c>
       <c r="D45">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">332k [SS6]</t>
+          <t xml:space="preserve">4.7k [CO3 IO6 SS4]</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC1206FR-074K7L</t>
-        </is>
-      </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-074K7L</t>
+          <t xml:space="preserve">CL31B475KBHNNNE</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">Samsung Electro-Mechanics</t>
         </is>
       </c>
       <c r="D46">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7k [CO3 IO6 SS4]</t>
+          <t xml:space="preserve">4.7uF 50V X7R [IO1]</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">CL31B475KBHNNNE</t>
+          <t xml:space="preserve">C1206C474K5RACTU</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samsung Electro-Mechanics</t>
+          <t xml:space="preserve">KEMET</t>
         </is>
       </c>
       <c r="D47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t xml:space="preserve">4.7uF 50V X7R [IO1]</t>
+          <t xml:space="preserve">470nF 50V X7R [SS2]</t>
         </is>
       </c>
     </row>
     <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603-MFR-25FBF52-470R</t>
+        </is>
+      </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1206C474K5RACTU</t>
+          <t xml:space="preserve">MFR-25FBF52-470R</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t xml:space="preserve">KEMET</t>
+          <t xml:space="preserve">Yageo</t>
         </is>
       </c>
       <c r="D48">
@@ -1158,19 +1158,19 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">470nF 50V X7R [SS2]</t>
+          <t xml:space="preserve">470R [PH2]</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-MFR-25FBF52-470R</t>
+          <t xml:space="preserve">603-RC1206FR-07470RL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">MFR-25FBF52-470R</t>
+          <t xml:space="preserve">RC1206FR-07470RL</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1179,23 +1179,23 @@
         </is>
       </c>
       <c r="D49">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t xml:space="preserve">470R [PH2]</t>
+          <t xml:space="preserve">470R [IO4]</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-RC1206FR-07470RL</t>
+          <t xml:space="preserve">603-RC1206FR-0747KL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-07470RL</t>
+          <t xml:space="preserve">RC1206FR-0747KL</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1204,23 +1204,23 @@
         </is>
       </c>
       <c r="D50">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">470R [IO4]</t>
+          <t xml:space="preserve">47k [SS1]</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-RC1206FR-0747KL</t>
+          <t xml:space="preserve">603-MFR-25FBF52-47R</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-0747KL</t>
+          <t xml:space="preserve">MFR-25FBF52-47R</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1229,23 +1229,23 @@
         </is>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">47k [SS1]</t>
+          <t xml:space="preserve">47R [PH3]</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-MFR-25FBF52-47R</t>
+          <t xml:space="preserve">603-RC1206FR-0747RL</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">MFR-25FBF52-47R</t>
+          <t xml:space="preserve">RC1206FR-0747RL</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1254,23 +1254,23 @@
         </is>
       </c>
       <c r="D52">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">47R [PH3]</t>
+          <t xml:space="preserve">47R [IO4]</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-RC1206FR-0747RL</t>
+          <t xml:space="preserve">603-RC1206FR-0749R9L</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-0747RL</t>
+          <t xml:space="preserve">RC1206FR-0749R9L</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1283,49 +1283,49 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">47R [IO4]</t>
+          <t xml:space="preserve">49.9R [CO4]</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">603-RC1206FR-0749R9L</t>
+          <t xml:space="preserve">576-0451004.MRL</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-0749R9L</t>
+          <t xml:space="preserve">0451004.MRL</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">Littelfuse</t>
         </is>
       </c>
       <c r="D54">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">49.9R [CO4]</t>
+          <t xml:space="preserve">4A [CO1]</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">576-0451004.MRL</t>
+          <t xml:space="preserve">603-RC1206FR-07680RL</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">0451004.MRL</t>
+          <t xml:space="preserve">RC1206FR-07680RL</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Littelfuse</t>
+          <t xml:space="preserve">Yageo</t>
         </is>
       </c>
       <c r="D55">
@@ -1333,24 +1333,19 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">4A [CO1]</t>
+          <t xml:space="preserve">680R [SS1]</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC1206FR-07680RL</t>
-        </is>
-      </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-07680RL</t>
+          <t xml:space="preserve">C1210C683KBRACTU</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">KEMET</t>
         </is>
       </c>
       <c r="D56">
@@ -1358,64 +1353,64 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">680R [SS1]</t>
+          <t xml:space="preserve">68nF 630V X7R [SS1]</t>
         </is>
       </c>
     </row>
     <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">603-RC1206FR-078K06L</t>
+        </is>
+      </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">C1210C683KBRACTU</t>
+          <t xml:space="preserve">RC1206FR-078K06L</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t xml:space="preserve">KEMET</t>
+          <t xml:space="preserve">Yageo</t>
         </is>
       </c>
       <c r="D57">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t xml:space="preserve">68nF 630V X7R [SS1]</t>
+          <t xml:space="preserve">8.06k [SS2]</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">603-RC1206FR-078K06L</t>
-        </is>
-      </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">RC1206FR-078K06L</t>
+          <t xml:space="preserve">ACS770LCB-100U-PFF-T</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yageo</t>
+          <t xml:space="preserve">Allegro MicroSystems</t>
         </is>
       </c>
       <c r="D58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">8.06k [SS2]</t>
+          <t xml:space="preserve">ACS770LCB-100U-PFF-T [SS1]</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACS770LCB-100U-PFF-T</t>
+          <t xml:space="preserve">68016-136HLF</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allegro MicroSystems</t>
+          <t xml:space="preserve">Amphenol FCI</t>
         </is>
       </c>
       <c r="D59">
@@ -1423,19 +1418,24 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">ACS770LCB-100U-PFF-T [SS1]</t>
+          <t xml:space="preserve">AD HAT terminal [PH1]</t>
         </is>
       </c>
     </row>
     <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">229-SH-7010MC</t>
+        </is>
+      </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">68016-136HLF</t>
+          <t xml:space="preserve">SH-7010MC</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amphenol FCI</t>
+          <t xml:space="preserve">Nidec Copal</t>
         </is>
       </c>
       <c r="D60">
@@ -1443,24 +1443,24 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">AD HAT terminal [PH1]</t>
+          <t xml:space="preserve">ADDR [SS1]</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">229-SH-7010MC</t>
+          <t xml:space="preserve">651-1844278</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">SH-7010MC</t>
+          <t xml:space="preserve">1844278</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nidec Copal</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D61">
@@ -1468,69 +1468,64 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">ADDR [SS1]</t>
+          <t xml:space="preserve">ANALOG OUT [IO1]</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844278</t>
+          <t xml:space="preserve">769-AQW212</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844278</t>
+          <t xml:space="preserve">AQW212</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Panasonic</t>
         </is>
       </c>
       <c r="D62">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANALOG OUT [IO1]</t>
+          <t xml:space="preserve">AQW212 [IO2]</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">769-AQW212</t>
+          <t xml:space="preserve">621-B340A-F</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQW212</t>
+          <t xml:space="preserve">B340A-13-F</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Panasonic</t>
+          <t xml:space="preserve">Diodes Incorporated</t>
         </is>
       </c>
       <c r="D63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">AQW212 [IO2]</t>
+          <t xml:space="preserve">B340A [SS1]</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">621-B340A-F</t>
-        </is>
-      </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">B340A-13-F</t>
+          <t xml:space="preserve">BAT54-7-F</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1543,14 +1538,14 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t xml:space="preserve">B340A [SS1]</t>
+          <t xml:space="preserve">BAT54 [SS1]</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAT54-7-F</t>
+          <t xml:space="preserve">BAT54S-7-F</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -1559,23 +1554,23 @@
         </is>
       </c>
       <c r="D65">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAT54 [SS1]</t>
+          <t xml:space="preserve">BAT54S [IO12]</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAT54S-7-F</t>
+          <t xml:space="preserve">BLM31PG391SN1L</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diodes Incorporated</t>
+          <t xml:space="preserve">Murata</t>
         </is>
       </c>
       <c r="D66">
@@ -1583,39 +1578,44 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">BAT54S [IO12]</t>
+          <t xml:space="preserve">BLM31PG391SN1L [CC8 SE4]</t>
         </is>
       </c>
     </row>
     <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">651-1953732</t>
+        </is>
+      </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLM31PG391SN1L</t>
+          <t xml:space="preserve">1953732</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Murata</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D67">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">BLM31PG391SN1L [CC8 SE4]</t>
+          <t xml:space="preserve">CAN IN/OUT [SS1]</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1953732</t>
+          <t xml:space="preserve">651-1844236</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">1953732</t>
+          <t xml:space="preserve">1844236</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -1624,48 +1624,48 @@
         </is>
       </c>
       <c r="D68">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAN IN/OUT [SS1]</t>
+          <t xml:space="preserve">CAN2 [CC4]</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844236</t>
+          <t xml:space="preserve">200-TSW10307GS</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844236</t>
+          <t xml:space="preserve">TSW-103-07-G-S</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D69">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAN2 [CC4]</t>
+          <t xml:space="preserve">COIL SUPPLY [IO1 SS1]</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">CC56-12SURKWA</t>
+          <t xml:space="preserve">ES1J</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kingbright</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="D70">
@@ -1673,114 +1673,119 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">CC56-12SURKWA [SS1]</t>
+          <t xml:space="preserve">ES1J [SS1]</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">200-TSW10307GS</t>
-        </is>
-      </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-103-07-G-S</t>
+          <t xml:space="preserve">ES3J</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
+          <t xml:space="preserve">onsemi</t>
+        </is>
+      </c>
+      <c r="D71">
+        <v>1</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ES3J [SS1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">875-HI1206P121R-10</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HI1206P121R-10</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Laird</t>
+        </is>
+      </c>
+      <c r="D72">
+        <v>3</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HI1206P121R-10 [CO3]</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200-TSW10607GS</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TSW-106-07-G-S</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
           <t xml:space="preserve">Samtec</t>
         </is>
       </c>
-      <c r="D71">
-        <v>2</v>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t xml:space="preserve">COIL SUPPLY [IO1 SS1]</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ES1J</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">onsemi</t>
-        </is>
-      </c>
-      <c r="D72">
-        <v>1</v>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ES1J [SS1]</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ES3J</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">onsemi</t>
-        </is>
-      </c>
       <c r="D73">
         <v>1</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">ES3J [SS1]</t>
+          <t xml:space="preserve">ICSP [SS1]</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">875-HI1206P121R-10</t>
+          <t xml:space="preserve">200-TSW10608GSRA</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">HI1206P121R-10</t>
+          <t xml:space="preserve">TSW-106-08-G-S-RA</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laird</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D74">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">HI1206P121R-10 [CO3]</t>
+          <t xml:space="preserve">ICSP [CO1]</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW10607GS</t>
+          <t xml:space="preserve">651-1844317</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-106-07-G-S</t>
+          <t xml:space="preserve">1844317</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D75">
@@ -1788,49 +1793,49 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICSP [SS1]</t>
+          <t xml:space="preserve">IO [IO1]</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW10608GSRA</t>
+          <t xml:space="preserve">726-IPB107N20N3GATMA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-106-08-G-S-RA</t>
+          <t xml:space="preserve">IPB107N20N3GATMA1</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">Infineon</t>
         </is>
       </c>
       <c r="D76">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">ICSP [CO1]</t>
+          <t xml:space="preserve">IPB107N20N3G [SS4]</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844317</t>
+          <t xml:space="preserve">595-ISO1540DR</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844317</t>
+          <t xml:space="preserve">ISO1540DR</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="D77">
@@ -1838,44 +1843,44 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">IO [IO1]</t>
+          <t xml:space="preserve">ISO1540 [IO1]</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">726-IPB107N20N3GATMA</t>
+          <t xml:space="preserve">595-ISO1640DWR</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">IPB107N20N3GATMA1</t>
+          <t xml:space="preserve">ISO1640DWR</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Infineon</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="D78">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t xml:space="preserve">IPB107N20N3G [SS4]</t>
+          <t xml:space="preserve">ISO1640DWR [SS1]</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">595-ISO1540DR</t>
+          <t xml:space="preserve">595-ISOW1044DFMR</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO1540DR</t>
+          <t xml:space="preserve">ISOW1044DFMR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1884,23 +1889,23 @@
         </is>
       </c>
       <c r="D79">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO1540 [IO1]</t>
+          <t xml:space="preserve">ISOW1044 [CC4]</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">595-ISO1640DWR</t>
+          <t xml:space="preserve">595-ISOW1432DFMR</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO1640DWR</t>
+          <t xml:space="preserve">ISOW1432DFMR</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -1909,93 +1914,93 @@
         </is>
       </c>
       <c r="D80">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISO1640DWR [SS1]</t>
+          <t xml:space="preserve">ISOW1432 [SE2]</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">595-ISOW1044DFMR</t>
+          <t xml:space="preserve">673-JD0-0004NL</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1044DFMR</t>
+          <t xml:space="preserve">JD0-0004NL</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve">Pulse Electronics</t>
         </is>
       </c>
       <c r="D81">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1044 [CC4]</t>
+          <t xml:space="preserve">JD0-0004NL [CO1]</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-ISOW1432DFMR</t>
-        </is>
-      </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1432DFMR</t>
+          <t xml:space="preserve">LTST-C150KGKT</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve">Lite-On</t>
         </is>
       </c>
       <c r="D82">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1432 [SE2]</t>
+          <t xml:space="preserve">LED green [CO3 SE4 SS1]</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">673-JD0-0004NL</t>
+          <t xml:space="preserve">859-LTST-C150KRKT</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t xml:space="preserve">JD0-0004NL</t>
+          <t xml:space="preserve">LTST-C150KRKT</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pulse Electronics</t>
+          <t xml:space="preserve">Lite-On</t>
         </is>
       </c>
       <c r="D83">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">JD0-0004NL [CO1]</t>
+          <t xml:space="preserve">LED red [IO4 SS1]</t>
         </is>
       </c>
     </row>
     <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">859-LTST-C150YKT</t>
+        </is>
+      </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t xml:space="preserve">LTST-C150KGKT</t>
+          <t xml:space="preserve">LTST-C150YKT</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2004,78 +2009,78 @@
         </is>
       </c>
       <c r="D84">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED green [CO3 SE4 SS3]</t>
+          <t xml:space="preserve">LED yellow [CC4 SE4]</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">859-LTST-C150KRKT</t>
+          <t xml:space="preserve">595-LM393BIDR</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t xml:space="preserve">LTST-C150KRKT</t>
+          <t xml:space="preserve">LM393BIDR</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lite-On</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="D85">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED red [IO4 SS1]</t>
+          <t xml:space="preserve">LM393B [SS1]</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">859-LTST-C150YKT</t>
+          <t xml:space="preserve">863-MC78L05ACHT1G</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t xml:space="preserve">LTST-C150YKT</t>
+          <t xml:space="preserve">MC78L05ACHT1G</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lite-On</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="D86">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">LED yellow [CC4 SE4]</t>
+          <t xml:space="preserve">MC78L05 [IO1]</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">595-LM393BIDR</t>
+          <t xml:space="preserve">579-MCP1826S-3302EDB</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">LM393BIDR</t>
+          <t xml:space="preserve">MCP1826S-3302E/DB</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D87">
@@ -2083,24 +2088,24 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t xml:space="preserve">LM393B [SS1]</t>
+          <t xml:space="preserve">MCP1826S-3302E/DB [CO1]</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">700-MAX7219CWG</t>
+          <t xml:space="preserve">579-MCP2562FD-E/P</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAX7219CWG+</t>
+          <t xml:space="preserve">MCP2562FD-E/P</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analog Devices</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D88">
@@ -2108,24 +2113,24 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t xml:space="preserve">MAX7219CWG+ [SS1]</t>
+          <t xml:space="preserve">MCP2562FD-E/P [SS1]</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">863-MC78L05ACHT1G</t>
+          <t xml:space="preserve">579-MCP3426A0E/SN</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t xml:space="preserve">MC78L05ACHT1G</t>
+          <t xml:space="preserve">MCP3426A0-E/SN</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t xml:space="preserve">onsemi</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D89">
@@ -2133,19 +2138,19 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">MC78L05 [IO1]</t>
+          <t xml:space="preserve">MCP3426A0-E/SN [SS1]</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP1826S-3302EDB</t>
+          <t xml:space="preserve">579-MCP3426A1-E/SN</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP1826S-3302E/DB</t>
+          <t xml:space="preserve">MCP3426A1-E/SN</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2158,19 +2163,19 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP1826S-3302E/DB [CO1]</t>
+          <t xml:space="preserve">MCP3426A1-E/SN [SS1]</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP2562FD-E/P</t>
+          <t xml:space="preserve">579-MCP4725A0TECH</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP2562FD-E/P</t>
+          <t xml:space="preserve">MCP4725A0T-E/CH</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -2179,28 +2184,28 @@
         </is>
       </c>
       <c r="D91">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP2562FD-E/P [SS1]</t>
+          <t xml:space="preserve">MCP4725A0T-E/CH [SS2]</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP3426A0E/SN</t>
+          <t xml:space="preserve">579-MCP4728-E/UN</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP3426A0-E/SN</t>
+          <t xml:space="preserve">MCP4728-E/UN</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">Microchip</t>
         </is>
       </c>
       <c r="D92">
@@ -2208,24 +2213,24 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP3426A0-E/SN [SS1]</t>
+          <t xml:space="preserve">MCP4728 [IO1]</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP3426A1-E/SN</t>
+          <t xml:space="preserve">651-1844249</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP3426A1-E/SN</t>
+          <t xml:space="preserve">1844249</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D93">
@@ -2233,74 +2238,74 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP3426A1-E/SN [SS1]</t>
+          <t xml:space="preserve">MEAN WELL [SS1]</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP4725A0TECH</t>
+          <t xml:space="preserve">863-MMBT2907ALT1G</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP4725A0T-E/CH</t>
+          <t xml:space="preserve">MMBT2907ALT1G</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="D94">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP4725A0T-E/CH [SS2]</t>
+          <t xml:space="preserve">MMBT2907A [SS1]</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-MCP4728-E/UN</t>
+          <t xml:space="preserve">863-NUP2105LT1G</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP4728-E/UN</t>
+          <t xml:space="preserve">NUP2105LT1G</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip</t>
+          <t xml:space="preserve">onsemi</t>
         </is>
       </c>
       <c r="D95">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP4728 [IO1]</t>
+          <t xml:space="preserve">NUP2105L [CC4 SS1]</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844249</t>
+          <t xml:space="preserve">595-OPA4171AIDR</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844249</t>
+          <t xml:space="preserve">OPA4171AIDR</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="D96">
@@ -2308,24 +2313,24 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">MEAN WELL [SS1]</t>
+          <t xml:space="preserve">OPA4171 [IO1]</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">863-MMBT2907ALT1G</t>
+          <t xml:space="preserve">710-61201021621</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMBT2907ALT1G</t>
+          <t xml:space="preserve">61201021621</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">onsemi</t>
+          <t xml:space="preserve">Wurth Elektronik</t>
         </is>
       </c>
       <c r="D97">
@@ -2333,49 +2338,49 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">MMBT2907A [SS1]</t>
+          <t xml:space="preserve">Pi pins 31-40 [PH1]</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">863-NUP2105LT1G</t>
+          <t xml:space="preserve">579-PIC18F47Q84-I/PT</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUP2105LT1G</t>
+          <t xml:space="preserve">PIC18F47Q84-I/PT</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">onsemi</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D98">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUP2105L [CC4 SS1]</t>
+          <t xml:space="preserve">PIC18F47Q84-I/PT [SS1]</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">595-OPA4171AIDR</t>
+          <t xml:space="preserve">579-2MK1024MCM064IPT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPA4171AIDR</t>
+          <t xml:space="preserve">PIC32MK1024MCM064-I/PT</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Texas Instruments</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D99">
@@ -2383,24 +2388,24 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">OPA4171 [IO1]</t>
+          <t xml:space="preserve">PIC32MK1024MCM064-I/PT [CO1]</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">710-61201021621</t>
+          <t xml:space="preserve">651-1715721</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">61201021621</t>
+          <t xml:space="preserve">1715721</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wurth Elektronik</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D100">
@@ -2408,24 +2413,24 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pi pins 31-40 [PH1]</t>
+          <t xml:space="preserve">PROBE A B [PH1]</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-PIC18F47Q84-I/PT</t>
+          <t xml:space="preserve">919-R-78E5.0-1.0</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC18F47Q84-I/PT</t>
+          <t xml:space="preserve">R-78E5.0-1.0</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">RECOM</t>
         </is>
       </c>
       <c r="D101">
@@ -2433,49 +2438,49 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC18F47Q84-I/PT [SS1]</t>
+          <t xml:space="preserve">R-78E5.0-1.0 [SS1]</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-2MK1024MCM064IPT</t>
+          <t xml:space="preserve">200-ESQ10314GD</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC32MK1024MCM064-I/PT</t>
+          <t xml:space="preserve">ESQ-103-14-G-D</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D102">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC32MK1024MCM064-I/PT [CO1]</t>
+          <t xml:space="preserve">RACK 12V [CC1 IO1 SE1]</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1715721</t>
+          <t xml:space="preserve">200-TSW10307GD</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">1715721</t>
+          <t xml:space="preserve">TSW-103-07-G-D</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D103">
@@ -2483,24 +2488,24 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROBE A B [PH1]</t>
+          <t xml:space="preserve">RACK 12V [CO1]</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">919-R-78E5.0-1.0</t>
+          <t xml:space="preserve">651-1844294</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">R-78E5.0-1.0</t>
+          <t xml:space="preserve">1844294</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">RECOM</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D104">
@@ -2508,49 +2513,44 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">R-78E5.0-1.0 [SS1]</t>
+          <t xml:space="preserve">RELAY [IO1]</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-ESQ10314GD</t>
+          <t xml:space="preserve">947-SM712.TCT</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESQ-103-14-G-D</t>
+          <t xml:space="preserve">SM712.TCT</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">Semtech</t>
         </is>
       </c>
       <c r="D105">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">RACK 12V [CC1 IO1 SE1]</t>
+          <t xml:space="preserve">SM712 [SE2]</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t xml:space="preserve">200-TSW10307GD</t>
-        </is>
-      </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-103-07-G-D</t>
+          <t xml:space="preserve">SMAZ15-13-F</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">Diodes Incorporated</t>
         </is>
       </c>
       <c r="D106">
@@ -2558,119 +2558,124 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">RACK 12V [CO1]</t>
+          <t xml:space="preserve">SMAZ15 [SS1]</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844294</t>
+          <t xml:space="preserve">947-SMBJ15A</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844294</t>
+          <t xml:space="preserve">SMBJ15A</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Littelfuse</t>
         </is>
       </c>
       <c r="D107">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t xml:space="preserve">RELAY [IO1]</t>
+          <t xml:space="preserve">SMBJ15A [CO1 SS1]</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">947-SM712.TCT</t>
+          <t xml:space="preserve">511-ST3232BDR</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">SM712.TCT</t>
+          <t xml:space="preserve">ST3232BDR</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Semtech</t>
+          <t xml:space="preserve">STMicroelectronics</t>
         </is>
       </c>
       <c r="D108">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">SM712 [SE2]</t>
+          <t xml:space="preserve">ST3232B [SE1]</t>
         </is>
       </c>
     </row>
     <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">200-ESQ12014GD</t>
+        </is>
+      </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMAZ15-13-F</t>
+          <t xml:space="preserve">ESQ-120-14-G-D</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Diodes Incorporated</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D109">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMAZ15 [SS1]</t>
+          <t xml:space="preserve">STACK BUS [CC1 IO1 SE1]</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">947-SMBJ15A</t>
+          <t xml:space="preserve">200-TSW12007GD</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMBJ15A</t>
+          <t xml:space="preserve">TSW-120-07-G-D</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Littelfuse</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D110">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMBJ15A [CO1 SS1]</t>
+          <t xml:space="preserve">STACK BUS [CO1]</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">511-ST3232BDR</t>
+          <t xml:space="preserve">781-SUD50P04-08-GE3</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST3232BDR</t>
+          <t xml:space="preserve">SUD50P04-08-GE3</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">STMicroelectronics</t>
+          <t xml:space="preserve">Vishay</t>
         </is>
       </c>
       <c r="D111">
@@ -2678,44 +2683,44 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST3232B [SE1]</t>
+          <t xml:space="preserve">SUD50P04-08 [CO1]</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-ESQ12014GD</t>
+          <t xml:space="preserve">495-TDN5-2411WI</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESQ-120-14-G-D</t>
+          <t xml:space="preserve">TDN 5-2411WI</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">TRACO Power</t>
         </is>
       </c>
       <c r="D112">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">STACK BUS [CC1 IO1 SE1]</t>
+          <t xml:space="preserve">TDN 5-2411WI [CO1]</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW12007GD</t>
+          <t xml:space="preserve">200-TSW10207GS</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-120-07-G-D</t>
+          <t xml:space="preserve">TSW-102-07-G-S</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -2724,28 +2729,23 @@
         </is>
       </c>
       <c r="D113">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">STACK BUS [CO1]</t>
+          <t xml:space="preserve">TERM [CC6 SE2 SS1]</t>
         </is>
       </c>
     </row>
     <row r="114">
-      <c r="A114" t="inlineStr">
-        <is>
-          <t xml:space="preserve">781-SUD50P04-08-GE3</t>
-        </is>
-      </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUD50P04-08-GE3</t>
+          <t xml:space="preserve">TLP240A(F)</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vishay</t>
+          <t xml:space="preserve">Toshiba</t>
         </is>
       </c>
       <c r="D114">
@@ -2753,24 +2753,24 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUD50P04-08 [CO1]</t>
+          <t xml:space="preserve">TLP240A [SS1]</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">495-TDN5-2411WI</t>
+          <t xml:space="preserve">200-TSW10308GSRA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">TDN 5-2411WI</t>
+          <t xml:space="preserve">TSW-103-08-G-S-RA</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t xml:space="preserve">TRACO Power</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D115">
@@ -2778,150 +2778,80 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t xml:space="preserve">TDN 5-2411WI [CO1]</t>
+          <t xml:space="preserve">UART [CO1]</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW10207GS</t>
+          <t xml:space="preserve">595-UCC12050DVE</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-102-07-G-S</t>
+          <t xml:space="preserve">UCC12050DVE</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">Texas Instruments</t>
         </is>
       </c>
       <c r="D116">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">TERM [CC6 SE2 SS1]</t>
+          <t xml:space="preserve">UCC12050DVE [SS1]</t>
         </is>
       </c>
     </row>
     <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">78-VOM1271T</t>
+        </is>
+      </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLP240A(F)</t>
+          <t xml:space="preserve">VOM1271T</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Toshiba</t>
+          <t xml:space="preserve">Vishay</t>
         </is>
       </c>
       <c r="D117">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t xml:space="preserve">TLP240A [SS1]</t>
+          <t xml:space="preserve">VOM1271T [SS2]</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW10308GSRA</t>
+          <t xml:space="preserve">950-W6100L</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-103-08-G-S-RA</t>
+          <t xml:space="preserve">W6100L</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">WIZnet</t>
         </is>
       </c>
       <c r="D118">
         <v>1</v>
       </c>
       <c r="E118" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UART [CO1]</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-UCC12050DVE</t>
-        </is>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UCC12050DVE</t>
-        </is>
-      </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Texas Instruments</t>
-        </is>
-      </c>
-      <c r="D119">
-        <v>1</v>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t xml:space="preserve">UCC12050DVE [SS1]</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">78-VOM1271T</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VOM1271T</t>
-        </is>
-      </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Vishay</t>
-        </is>
-      </c>
-      <c r="D120">
-        <v>2</v>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t xml:space="preserve">VOM1271T [SS2]</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">950-W6100L</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">W6100L</t>
-        </is>
-      </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WIZnet</t>
-        </is>
-      </c>
-      <c r="D121">
-        <v>1</v>
-      </c>
-      <c r="E121" t="inlineStr">
         <is>
           <t xml:space="preserve">W6100-L [CO1]</t>
         </is>

</xml_diff>

<commit_message>
Mouser order: IPB107N20N3 G (ATMA1 reel code out of stock)
Same Infineon part; Mouser has stock under the device name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -1798,14 +1798,9 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t xml:space="preserve">726-IPB107N20N3GATMA</t>
-        </is>
-      </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">IPB107N20N3GATMA1</t>
+          <t xml:space="preserve">IPB107N20N3 G</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">

</xml_diff>

<commit_message>
Mouser order: MCP1826ST-3302E/DB (reel code; MCP1826S-3302E/DB out of stock)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -2063,14 +2063,9 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">579-MCP1826S-3302EDB</t>
-        </is>
-      </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t xml:space="preserve">MCP1826S-3302E/DB</t>
+          <t xml:space="preserve">MCP1826ST-3302E/DB</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">

</xml_diff>

<commit_message>
Rev B / rev A order: ISOW1044BDFMR (ISOW1044DFMR out of stock)
Same TI part, package and pinout with basic instead of reinforced
isolation; the CAN buses are low-voltage and isolated against ground
loops, not for safety. Field-only change on can-card (and the reference
can-controller); order lists regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -1868,14 +1868,9 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t xml:space="preserve">595-ISOW1044DFMR</t>
-        </is>
-      </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1044DFMR</t>
+          <t xml:space="preserve">ISOW1044BDFMR</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -1888,7 +1883,7 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t xml:space="preserve">ISOW1044 [CC4]</t>
+          <t xml:space="preserve">ISOW1044B [CC4]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mouser cart: SQD50P04-09L P-FET, Diotec P6SMBJ15A TVS
Out of stock: Vishay SUD50P04-08-GE3 (core Q1) -> SQD50P04-09L_GE3 and
Littelfuse SMBJ15A (12 V input TVS) -> Diotec P6SMBJ15A, same footprints,
in core, can-ssr and the can-controller/pic-module references. Logged in
docs/rev-b-changes.md; order lists regenerated. The cart as ordered is
docs/orders/mouser-cart-2026-10-12.xls.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/orders/mouser-revA-simple.xlsx
+++ b/docs/orders/mouser-revA-simple.xlsx
@@ -2303,44 +2303,39 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
-        <is>
-          <t xml:space="preserve">710-61201021621</t>
-        </is>
-      </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t xml:space="preserve">61201021621</t>
+          <t xml:space="preserve">P6SMBJ15A</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wurth Elektronik</t>
+          <t xml:space="preserve">Diotec Semiconductor</t>
         </is>
       </c>
       <c r="D97">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pi pins 31-40 [PH1]</t>
+          <t xml:space="preserve">P6SMBJ15A [CO1 SS1]</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-PIC18F47Q84-I/PT</t>
+          <t xml:space="preserve">710-61201021621</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC18F47Q84-I/PT</t>
+          <t xml:space="preserve">61201021621</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Microchip Technology</t>
+          <t xml:space="preserve">Wurth Elektronik</t>
         </is>
       </c>
       <c r="D98">
@@ -2348,19 +2343,19 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC18F47Q84-I/PT [SS1]</t>
+          <t xml:space="preserve">Pi pins 31-40 [PH1]</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">579-2MK1024MCM064IPT</t>
+          <t xml:space="preserve">579-PIC18F47Q84-I/PT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC32MK1024MCM064-I/PT</t>
+          <t xml:space="preserve">PIC18F47Q84-I/PT</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -2373,24 +2368,24 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t xml:space="preserve">PIC32MK1024MCM064-I/PT [CO1]</t>
+          <t xml:space="preserve">PIC18F47Q84-I/PT [SS1]</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1715721</t>
+          <t xml:space="preserve">579-2MK1024MCM064IPT</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t xml:space="preserve">1715721</t>
+          <t xml:space="preserve">PIC32MK1024MCM064-I/PT</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Microchip Technology</t>
         </is>
       </c>
       <c r="D100">
@@ -2398,24 +2393,24 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">PROBE A B [PH1]</t>
+          <t xml:space="preserve">PIC32MK1024MCM064-I/PT [CO1]</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">919-R-78E5.0-1.0</t>
+          <t xml:space="preserve">651-1715721</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t xml:space="preserve">R-78E5.0-1.0</t>
+          <t xml:space="preserve">1715721</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t xml:space="preserve">RECOM</t>
+          <t xml:space="preserve">Phoenix Contact</t>
         </is>
       </c>
       <c r="D101">
@@ -2423,44 +2418,44 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">R-78E5.0-1.0 [SS1]</t>
+          <t xml:space="preserve">PROBE A B [PH1]</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-ESQ10314GD</t>
+          <t xml:space="preserve">919-R-78E5.0-1.0</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESQ-103-14-G-D</t>
+          <t xml:space="preserve">R-78E5.0-1.0</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">RECOM</t>
         </is>
       </c>
       <c r="D102">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">RACK 12V [CC1 IO1 SE1]</t>
+          <t xml:space="preserve">R-78E5.0-1.0 [SS1]</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW10307GD</t>
+          <t xml:space="preserve">200-ESQ10314GD</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-103-07-G-D</t>
+          <t xml:space="preserve">ESQ-103-14-G-D</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2469,28 +2464,28 @@
         </is>
       </c>
       <c r="D103">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t xml:space="preserve">RACK 12V [CO1]</t>
+          <t xml:space="preserve">RACK 12V [CC1 IO1 SE1]</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">651-1844294</t>
+          <t xml:space="preserve">200-TSW10307GD</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t xml:space="preserve">1844294</t>
+          <t xml:space="preserve">TSW-103-07-G-D</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Phoenix Contact</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D104">
@@ -2498,94 +2493,89 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t xml:space="preserve">RELAY [IO1]</t>
+          <t xml:space="preserve">RACK 12V [CO1]</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t xml:space="preserve">651-1844294</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1844294</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phoenix Contact</t>
+        </is>
+      </c>
+      <c r="D105">
+        <v>1</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RELAY [IO1]</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
           <t xml:space="preserve">947-SM712.TCT</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t xml:space="preserve">SM712.TCT</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t xml:space="preserve">Semtech</t>
         </is>
       </c>
-      <c r="D105">
+      <c r="D106">
         <v>2</v>
       </c>
-      <c r="E105" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t xml:space="preserve">SM712 [SE2]</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="B106" t="inlineStr">
+    <row r="107">
+      <c r="B107" t="inlineStr">
         <is>
           <t xml:space="preserve">SMAZ15-13-F</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t xml:space="preserve">Diodes Incorporated</t>
         </is>
       </c>
-      <c r="D106">
-        <v>1</v>
-      </c>
-      <c r="E106" t="inlineStr">
+      <c r="D107">
+        <v>1</v>
+      </c>
+      <c r="E107" t="inlineStr">
         <is>
           <t xml:space="preserve">SMAZ15 [SS1]</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">947-SMBJ15A</t>
-        </is>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SMBJ15A</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Littelfuse</t>
-        </is>
-      </c>
-      <c r="D107">
-        <v>2</v>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">SMBJ15A [CO1 SS1]</t>
-        </is>
-      </c>
-    </row>
     <row r="108">
-      <c r="A108" t="inlineStr">
-        <is>
-          <t xml:space="preserve">511-ST3232BDR</t>
-        </is>
-      </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST3232BDR</t>
+          <t xml:space="preserve">SQD50P04-09L_GE3</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t xml:space="preserve">STMicroelectronics</t>
+          <t xml:space="preserve">Vishay</t>
         </is>
       </c>
       <c r="D108">
@@ -2593,44 +2583,44 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t xml:space="preserve">ST3232B [SE1]</t>
+          <t xml:space="preserve">SQD50P04-09L [CO1]</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-ESQ12014GD</t>
+          <t xml:space="preserve">511-ST3232BDR</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t xml:space="preserve">ESQ-120-14-G-D</t>
+          <t xml:space="preserve">ST3232BDR</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samtec</t>
+          <t xml:space="preserve">STMicroelectronics</t>
         </is>
       </c>
       <c r="D109">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">STACK BUS [CC1 IO1 SE1]</t>
+          <t xml:space="preserve">ST3232B [SE1]</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">200-TSW12007GD</t>
+          <t xml:space="preserve">200-ESQ12014GD</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t xml:space="preserve">TSW-120-07-G-D</t>
+          <t xml:space="preserve">ESQ-120-14-G-D</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -2639,28 +2629,28 @@
         </is>
       </c>
       <c r="D110">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">STACK BUS [CO1]</t>
+          <t xml:space="preserve">STACK BUS [CC1 IO1 SE1]</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">781-SUD50P04-08-GE3</t>
+          <t xml:space="preserve">200-TSW12007GD</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUD50P04-08-GE3</t>
+          <t xml:space="preserve">TSW-120-07-G-D</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vishay</t>
+          <t xml:space="preserve">Samtec</t>
         </is>
       </c>
       <c r="D111">
@@ -2668,7 +2658,7 @@
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">SUD50P04-08 [CO1]</t>
+          <t xml:space="preserve">STACK BUS [CO1]</t>
         </is>
       </c>
     </row>

</xml_diff>